<commit_message>
Update BOM dual syringe pump.xlsx
</commit_message>
<xml_diff>
--- a/Open Syringe Pump/dual syringepump build and test/BOM dual syringe pump.xlsx
+++ b/Open Syringe Pump/dual syringepump build and test/BOM dual syringe pump.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twenzel/Documents/GitHub/OpenMicrofluidics/dual syringepump build and test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twenzel/Documents/GitHub/OpenMicrofluidics/Open Syringe Pump/dual syringepump build and test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCBFEF5-6AD1-0147-BE53-38B004277B07}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2712CE-DEFC-0B48-BCA4-F437A33CF582}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12520" yWindow="3640" windowWidth="20720" windowHeight="16740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="279">
   <si>
     <r>
       <rPr>
@@ -3004,6 +3004,9 @@
   </si>
   <si>
     <t>bought</t>
+  </si>
+  <si>
+    <t>which do I have?</t>
   </si>
 </sst>
 </file>
@@ -3493,22 +3496,34 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3523,19 +3538,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4458,10 +4461,10 @@
       <c r="B3" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="75" t="s">
+      <c r="C3" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="75"/>
+      <c r="D3" s="89"/>
       <c r="E3" s="22">
         <v>35</v>
       </c>
@@ -4483,10 +4486,10 @@
       <c r="B4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="76" t="s">
+      <c r="C4" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="76"/>
+      <c r="D4" s="80"/>
       <c r="E4" s="16">
         <v>9.89</v>
       </c>
@@ -4508,10 +4511,10 @@
       <c r="B5" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="76" t="s">
+      <c r="C5" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="76"/>
+      <c r="D5" s="80"/>
       <c r="E5" s="16">
         <v>60</v>
       </c>
@@ -4559,10 +4562,10 @@
       <c r="B7" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="76" t="s">
+      <c r="C7" s="80" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="76"/>
+      <c r="D7" s="80"/>
       <c r="E7" s="16">
         <v>18.5</v>
       </c>
@@ -4656,10 +4659,10 @@
       <c r="B11" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="79">
+      <c r="C11" s="83">
         <v>237825</v>
       </c>
-      <c r="D11" s="79"/>
+      <c r="D11" s="83"/>
       <c r="E11" s="16">
         <v>9.9499999999999993</v>
       </c>
@@ -4683,10 +4686,10 @@
       <c r="B12" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="80" t="s">
+      <c r="C12" s="79" t="s">
         <v>97</v>
       </c>
-      <c r="D12" s="76"/>
+      <c r="D12" s="80"/>
       <c r="E12" s="59" t="s">
         <v>18</v>
       </c>
@@ -4710,10 +4713,10 @@
       <c r="B13" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="76" t="s">
+      <c r="C13" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="76"/>
+      <c r="D13" s="80"/>
       <c r="E13" s="16">
         <v>25</v>
       </c>
@@ -4735,10 +4738,10 @@
       <c r="B14" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="C14" s="81" t="s">
+      <c r="C14" s="85" t="s">
         <v>84</v>
       </c>
-      <c r="D14" s="82"/>
+      <c r="D14" s="86"/>
       <c r="E14" s="27">
         <v>32.869999999999997</v>
       </c>
@@ -4760,10 +4763,10 @@
       <c r="B15" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C15" s="80" t="s">
+      <c r="C15" s="79" t="s">
         <v>94</v>
       </c>
-      <c r="D15" s="76"/>
+      <c r="D15" s="80"/>
       <c r="E15" s="16">
         <v>10.68</v>
       </c>
@@ -4787,10 +4790,10 @@
       <c r="B16" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="80" t="s">
+      <c r="C16" s="79" t="s">
         <v>85</v>
       </c>
-      <c r="D16" s="76"/>
+      <c r="D16" s="80"/>
       <c r="E16" s="59">
         <v>5.62</v>
       </c>
@@ -4814,10 +4817,10 @@
       <c r="B17" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="83" t="s">
+      <c r="C17" s="87" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="84"/>
+      <c r="D17" s="88"/>
       <c r="E17" s="60">
         <v>0.56999999999999995</v>
       </c>
@@ -4839,10 +4842,10 @@
       <c r="B18" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="76" t="s">
+      <c r="C18" s="80" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="76"/>
+      <c r="D18" s="80"/>
       <c r="E18" s="59" t="s">
         <v>143</v>
       </c>
@@ -4866,10 +4869,10 @@
       <c r="B19" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="80" t="s">
+      <c r="C19" s="79" t="s">
         <v>86</v>
       </c>
-      <c r="D19" s="76"/>
+      <c r="D19" s="80"/>
       <c r="E19" s="16">
         <v>0.11</v>
       </c>
@@ -4893,10 +4896,10 @@
       <c r="B20" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="81" t="s">
+      <c r="C20" s="85" t="s">
         <v>87</v>
       </c>
-      <c r="D20" s="82"/>
+      <c r="D20" s="86"/>
       <c r="E20" s="27">
         <v>0.25</v>
       </c>
@@ -4918,10 +4921,10 @@
       <c r="B21" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="81" t="s">
+      <c r="C21" s="85" t="s">
         <v>88</v>
       </c>
-      <c r="D21" s="82"/>
+      <c r="D21" s="86"/>
       <c r="E21" s="27">
         <v>0.1</v>
       </c>
@@ -4943,10 +4946,10 @@
       <c r="B22" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="80" t="s">
+      <c r="C22" s="79" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="76"/>
+      <c r="D22" s="80"/>
       <c r="E22" s="16">
         <v>1.25</v>
       </c>
@@ -4970,10 +4973,10 @@
       <c r="B23" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="C23" s="79">
+      <c r="C23" s="83">
         <v>856</v>
       </c>
-      <c r="D23" s="79"/>
+      <c r="D23" s="83"/>
       <c r="E23" s="59">
         <v>3.75</v>
       </c>
@@ -4997,10 +5000,10 @@
       <c r="B24" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="80" t="s">
+      <c r="C24" s="79" t="s">
         <v>90</v>
       </c>
-      <c r="D24" s="76"/>
+      <c r="D24" s="80"/>
       <c r="E24" s="16">
         <v>0.15</v>
       </c>
@@ -5024,10 +5027,10 @@
       <c r="B25" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C25" s="79">
+      <c r="C25" s="83">
         <v>2222</v>
       </c>
-      <c r="D25" s="79"/>
+      <c r="D25" s="83"/>
       <c r="E25" s="16">
         <v>1</v>
       </c>
@@ -5051,10 +5054,10 @@
       <c r="B26" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="80" t="s">
+      <c r="C26" s="79" t="s">
         <v>91</v>
       </c>
-      <c r="D26" s="76"/>
+      <c r="D26" s="80"/>
       <c r="E26" s="16">
         <v>0.09</v>
       </c>
@@ -5138,10 +5141,10 @@
       <c r="B29" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="C29" s="80">
+      <c r="C29" s="79">
         <v>1952370</v>
       </c>
-      <c r="D29" s="76"/>
+      <c r="D29" s="80"/>
       <c r="E29" s="62">
         <v>18.95</v>
       </c>
@@ -5165,10 +5168,10 @@
       <c r="B30" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="85" t="s">
+      <c r="C30" s="76" t="s">
         <v>42</v>
       </c>
-      <c r="D30" s="85"/>
+      <c r="D30" s="76"/>
       <c r="E30" s="46">
         <v>0.43</v>
       </c>
@@ -5232,10 +5235,10 @@
       <c r="B33" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="C33" s="80" t="s">
+      <c r="C33" s="79" t="s">
         <v>93</v>
       </c>
-      <c r="D33" s="76"/>
+      <c r="D33" s="80"/>
       <c r="E33" s="59">
         <v>1.25</v>
       </c>
@@ -5259,10 +5262,10 @@
       <c r="B34" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="C34" s="79">
+      <c r="C34" s="83">
         <v>2094346</v>
       </c>
-      <c r="D34" s="79"/>
+      <c r="D34" s="83"/>
       <c r="E34" s="67">
         <v>6.9000000000000006E-2</v>
       </c>
@@ -5286,10 +5289,10 @@
       <c r="B35" s="62" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="79">
+      <c r="C35" s="83">
         <v>106797</v>
       </c>
-      <c r="D35" s="79"/>
+      <c r="D35" s="83"/>
       <c r="E35" s="67">
         <v>7.9000000000000001E-2</v>
       </c>
@@ -5313,10 +5316,10 @@
       <c r="B36" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="86">
+      <c r="C36" s="84">
         <v>106810</v>
       </c>
-      <c r="D36" s="86"/>
+      <c r="D36" s="84"/>
       <c r="E36" s="67">
         <v>7.9000000000000001E-2</v>
       </c>
@@ -5340,10 +5343,10 @@
       <c r="B37" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="C37" s="79">
+      <c r="C37" s="83">
         <v>38173</v>
       </c>
-      <c r="D37" s="79"/>
+      <c r="D37" s="83"/>
       <c r="E37" s="67">
         <v>9.9000000000000005E-2</v>
       </c>
@@ -5367,10 +5370,10 @@
       <c r="B38" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="C38" s="76">
+      <c r="C38" s="80">
         <v>51553</v>
       </c>
-      <c r="D38" s="76"/>
+      <c r="D38" s="80"/>
       <c r="E38" s="67">
         <v>5.8999999999999997E-2</v>
       </c>
@@ -5394,10 +5397,10 @@
       <c r="B39" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="C39" s="79">
+      <c r="C39" s="83">
         <v>40943</v>
       </c>
-      <c r="D39" s="79"/>
+      <c r="D39" s="83"/>
       <c r="E39" s="62">
         <v>5.8999999999999997E-2</v>
       </c>
@@ -5421,10 +5424,10 @@
       <c r="B40" s="62" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="76">
+      <c r="C40" s="80">
         <v>38165</v>
       </c>
-      <c r="D40" s="76"/>
+      <c r="D40" s="80"/>
       <c r="E40" s="62">
         <v>5.8999999999999997E-2</v>
       </c>
@@ -5448,10 +5451,10 @@
       <c r="B41" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="C41" s="86">
+      <c r="C41" s="84">
         <v>106850</v>
       </c>
-      <c r="D41" s="86"/>
+      <c r="D41" s="84"/>
       <c r="E41" s="67">
         <v>5.8999999999999997E-2</v>
       </c>
@@ -5475,10 +5478,10 @@
       <c r="B42" s="68" t="s">
         <v>54</v>
       </c>
-      <c r="C42" s="79">
+      <c r="C42" s="83">
         <v>106826</v>
       </c>
-      <c r="D42" s="79"/>
+      <c r="D42" s="83"/>
       <c r="E42" s="62">
         <v>6.5000000000000002E-2</v>
       </c>
@@ -5637,7 +5640,7 @@
       <c r="B48" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C48" s="87" t="s">
+      <c r="C48" s="81" t="s">
         <v>123</v>
       </c>
       <c r="D48" s="78"/>
@@ -5691,10 +5694,10 @@
       <c r="B50" s="62" t="s">
         <v>64</v>
       </c>
-      <c r="C50" s="80">
+      <c r="C50" s="79">
         <v>2135064</v>
       </c>
-      <c r="D50" s="76"/>
+      <c r="D50" s="80"/>
       <c r="E50" s="16">
         <v>2.4900000000000002</v>
       </c>
@@ -5718,7 +5721,7 @@
       <c r="B51" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C51" s="87" t="s">
+      <c r="C51" s="81" t="s">
         <v>99</v>
       </c>
       <c r="D51" s="78"/>
@@ -5742,10 +5745,10 @@
       <c r="B52" s="42" t="s">
         <v>67</v>
       </c>
-      <c r="C52" s="89" t="s">
+      <c r="C52" s="82" t="s">
         <v>101</v>
       </c>
-      <c r="D52" s="85"/>
+      <c r="D52" s="76"/>
       <c r="E52" s="46">
         <v>9.99</v>
       </c>
@@ -5790,10 +5793,10 @@
       <c r="B54" s="42" t="s">
         <v>69</v>
       </c>
-      <c r="C54" s="88" t="s">
+      <c r="C54" s="75" t="s">
         <v>102</v>
       </c>
-      <c r="D54" s="85"/>
+      <c r="D54" s="76"/>
       <c r="E54" s="45"/>
       <c r="F54" s="55">
         <v>5</v>
@@ -5811,10 +5814,10 @@
       <c r="B55" s="45" t="s">
         <v>70</v>
       </c>
-      <c r="C55" s="85" t="s">
+      <c r="C55" s="76" t="s">
         <v>71</v>
       </c>
-      <c r="D55" s="85"/>
+      <c r="D55" s="76"/>
       <c r="E55" s="45"/>
       <c r="F55" s="45"/>
       <c r="G55" s="45"/>
@@ -5830,10 +5833,10 @@
       <c r="B56" s="42" t="s">
         <v>74</v>
       </c>
-      <c r="C56" s="85" t="s">
+      <c r="C56" s="76" t="s">
         <v>75</v>
       </c>
-      <c r="D56" s="85"/>
+      <c r="D56" s="76"/>
       <c r="E56" s="45"/>
       <c r="F56" s="45"/>
       <c r="G56" s="45"/>
@@ -5849,6 +5852,51 @@
     </row>
   </sheetData>
   <mergeCells count="53">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
     <mergeCell ref="C54:D54"/>
     <mergeCell ref="C55:D55"/>
     <mergeCell ref="C56:D56"/>
@@ -5857,51 +5905,6 @@
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="C53:D53"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I31" r:id="rId1" xr:uid="{A02AF87C-9527-A047-9DFE-4A7472C1BB6D}"/>
@@ -6524,6 +6527,9 @@
       <c r="G28" s="72" t="s">
         <v>221</v>
       </c>
+      <c r="I28" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="29" spans="1:9" ht="17" x14ac:dyDescent="0.15">
       <c r="A29" s="72" t="s">

</xml_diff>